<commit_message>
Fix database integration and API routing
- Fix SportSelection button logic (operator precedence)
- Implement competitions API call in page.tsx
- Add error handling and loading states
- Display competitions from database dynamically
- Add validation for missing data

Database verified: 16 venues across 8 sports
All API routes tested and working
</commit_message>
<xml_diff>
--- a/public/databases/iconic-venues.xlsx
+++ b/public/databases/iconic-venues.xlsx
@@ -4,7 +4,13 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Formula 1" sheetId="1" r:id="rId1"/>
-    <sheet name="Football Stadiums" sheetId="2" r:id="rId2"/>
+    <sheet name="Football" sheetId="2" r:id="rId2"/>
+    <sheet name="Cricket" sheetId="3" r:id="rId3"/>
+    <sheet name="Tennis" sheetId="4" r:id="rId4"/>
+    <sheet name="Golf" sheetId="5" r:id="rId5"/>
+    <sheet name="Rugby" sheetId="6" r:id="rId6"/>
+    <sheet name="Olympic Venues" sheetId="7" r:id="rId7"/>
+    <sheet name="Boxing" sheetId="8" r:id="rId8"/>
   </sheets>
 </workbook>
 </file>
@@ -398,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X2"/>
+  <dimension ref="A1:Q4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -417,60 +423,39 @@
         <v>country</v>
       </c>
       <c r="F1" t="str">
-        <v>countryFlag</v>
+        <v>opened</v>
       </c>
       <c r="G1" t="str">
-        <v>opened</v>
+        <v>capacity</v>
       </c>
       <c r="H1" t="str">
-        <v>capacity</v>
+        <v>lat</v>
       </c>
       <c r="I1" t="str">
-        <v>lat</v>
+        <v>lng</v>
       </c>
       <c r="J1" t="str">
-        <v>lng</v>
+        <v>architect</v>
       </c>
       <c r="K1" t="str">
-        <v>architect</v>
+        <v>surface</v>
       </c>
       <c r="L1" t="str">
-        <v>surface</v>
+        <v>raceDistance</v>
       </c>
       <c r="M1" t="str">
-        <v>themePrimary</v>
+        <v>numberOfTurns</v>
       </c>
       <c r="N1" t="str">
-        <v>themeSecondary</v>
+        <v>nickname</v>
       </c>
       <c r="O1" t="str">
-        <v>themeAccent</v>
+        <v>famousFor</v>
       </c>
       <c r="P1" t="str">
-        <v>famousFor</v>
+        <v>iconicMoments</v>
       </c>
       <c r="Q1" t="str">
-        <v>iconicMoments</v>
-      </c>
-      <c r="R1" t="str">
-        <v>raceDistance</v>
-      </c>
-      <c r="S1" t="str">
-        <v>numberOfTurns</v>
-      </c>
-      <c r="T1" t="str">
-        <v>altitude</v>
-      </c>
-      <c r="U1" t="str">
-        <v>nickname</v>
-      </c>
-      <c r="V1" t="str">
-        <v>notableEvents</v>
-      </c>
-      <c r="W1" t="str">
-        <v>championshipHistory</v>
-      </c>
-      <c r="X1" t="str">
         <v>collectorNumber</v>
       </c>
     </row>
@@ -490,74 +475,159 @@
       <c r="E2" t="str">
         <v>Monaco</v>
       </c>
-      <c r="F2" t="str">
-        <v>🇲🇨</v>
+      <c r="F2">
+        <v>1929</v>
       </c>
       <c r="G2">
-        <v>1929</v>
+        <v>37000</v>
       </c>
       <c r="H2">
-        <v>37000</v>
+        <v>43.7347</v>
       </c>
       <c r="I2">
-        <v>43.7347</v>
-      </c>
-      <c r="J2">
         <v>7.4206</v>
       </c>
+      <c r="J2" t="str">
+        <v>Charles Leclerc</v>
+      </c>
       <c r="K2" t="str">
-        <v>Charles Leclerc</v>
-      </c>
-      <c r="L2" t="str">
         <v>Asphalt</v>
       </c>
-      <c r="M2" t="str">
-        <v>#1a1a1a</v>
+      <c r="L2">
+        <v>3.337</v>
+      </c>
+      <c r="M2">
+        <v>19</v>
       </c>
       <c r="N2" t="str">
-        <v>#c41e3a</v>
+        <v>Street Circuit in the Sky</v>
       </c>
       <c r="O2" t="str">
-        <v>#d4af37</v>
+        <v>Prestige,Street circuit,Glamour</v>
       </c>
       <c r="P2" t="str">
-        <v>Street circuit,Prestige,Casino</v>
-      </c>
-      <c r="Q2" t="str">
-        <v>Senna victory record|Leclerc home win 2024</v>
-      </c>
-      <c r="R2">
-        <v>3.337</v>
-      </c>
-      <c r="S2">
-        <v>19</v>
-      </c>
-      <c r="T2">
-        <v>65</v>
-      </c>
-      <c r="U2" t="str">
-        <v>Street Circuit in the Sky</v>
-      </c>
-      <c r="V2" t="str">
-        <v>F1 Championship|Monaco Grand Prix</v>
-      </c>
-      <c r="W2" t="str">
-        <v>Senna 6 times|Leclerc 2024</v>
-      </c>
-      <c r="X2">
+        <v>Senna victories|Leclerc home win 2024</v>
+      </c>
+      <c r="Q2">
         <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Formula 1</v>
+      </c>
+      <c r="B3" t="str">
+        <v>British Grand Prix</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Silverstone Circuit</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Northamptonshire</v>
+      </c>
+      <c r="E3" t="str">
+        <v>United Kingdom</v>
+      </c>
+      <c r="F3">
+        <v>1948</v>
+      </c>
+      <c r="G3">
+        <v>140000</v>
+      </c>
+      <c r="H3">
+        <v>52.0786</v>
+      </c>
+      <c r="I3">
+        <v>-1.0169</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Historic Design</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Asphalt</v>
+      </c>
+      <c r="L3">
+        <v>5.891</v>
+      </c>
+      <c r="M3">
+        <v>18</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Home of British Racing</v>
+      </c>
+      <c r="O3" t="str">
+        <v>Speed,Racing heritage,History</v>
+      </c>
+      <c r="P3" t="str">
+        <v>First F1 race 1950|Hamilton records</v>
+      </c>
+      <c r="Q3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Formula 1</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Italian Grand Prix</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Autodromo di Monza</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Monza</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Italy</v>
+      </c>
+      <c r="F4">
+        <v>1922</v>
+      </c>
+      <c r="G4">
+        <v>80000</v>
+      </c>
+      <c r="H4">
+        <v>45.6211</v>
+      </c>
+      <c r="I4">
+        <v>9.2819</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Historic</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Asphalt</v>
+      </c>
+      <c r="L4">
+        <v>5.793</v>
+      </c>
+      <c r="M4">
+        <v>11</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Temple of Speed</v>
+      </c>
+      <c r="O4" t="str">
+        <v>Speed,High speed,Tradition</v>
+      </c>
+      <c r="P4" t="str">
+        <v>Senna-Prost crash|Schumacher wins</v>
+      </c>
+      <c r="Q4">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:X2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:O5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -576,60 +646,39 @@
         <v>country</v>
       </c>
       <c r="F1" t="str">
-        <v>countryFlag</v>
+        <v>opened</v>
       </c>
       <c r="G1" t="str">
-        <v>opened</v>
+        <v>capacity</v>
       </c>
       <c r="H1" t="str">
-        <v>capacity</v>
+        <v>lat</v>
       </c>
       <c r="I1" t="str">
-        <v>lat</v>
+        <v>lng</v>
       </c>
       <c r="J1" t="str">
-        <v>lng</v>
+        <v>architect</v>
       </c>
       <c r="K1" t="str">
-        <v>architect</v>
+        <v>surface</v>
       </c>
       <c r="L1" t="str">
-        <v>surface</v>
+        <v>nickname</v>
       </c>
       <c r="M1" t="str">
-        <v>themePrimary</v>
+        <v>famousFor</v>
       </c>
       <c r="N1" t="str">
-        <v>themeSecondary</v>
+        <v>iconicMoments</v>
       </c>
       <c r="O1" t="str">
-        <v>themeAccent</v>
-      </c>
-      <c r="P1" t="str">
-        <v>famousFor</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>iconicMoments</v>
-      </c>
-      <c r="R1" t="str">
-        <v>altitude</v>
-      </c>
-      <c r="S1" t="str">
-        <v>nickname</v>
-      </c>
-      <c r="T1" t="str">
-        <v>notableEvents</v>
-      </c>
-      <c r="U1" t="str">
-        <v>championshipHistory</v>
-      </c>
-      <c r="V1" t="str">
         <v>collectorNumber</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Football Stadiums</v>
+        <v>Football</v>
       </c>
       <c r="B2" t="str">
         <v>Premier League</v>
@@ -643,61 +692,952 @@
       <c r="E2" t="str">
         <v>England</v>
       </c>
-      <c r="F2" t="str">
-        <v>🏴󠁧󠁢󠁥󠁮󠁧󠁿</v>
+      <c r="F2">
+        <v>1910</v>
       </c>
       <c r="G2">
-        <v>1910</v>
+        <v>74310</v>
       </c>
       <c r="H2">
-        <v>74310</v>
+        <v>53.4629</v>
       </c>
       <c r="I2">
-        <v>53.4629</v>
-      </c>
-      <c r="J2">
         <v>-2.2913</v>
       </c>
+      <c r="J2" t="str">
+        <v>Archibald Leitch</v>
+      </c>
       <c r="K2" t="str">
-        <v>Archibald Leitch</v>
+        <v>Grass</v>
       </c>
       <c r="L2" t="str">
+        <v>Theatre of Dreams</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Manchester United,History,Iconic</v>
+      </c>
+      <c r="N2" t="str">
+        <v>FA Cup wins|European victories</v>
+      </c>
+      <c r="O2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Football</v>
+      </c>
+      <c r="B3" t="str">
+        <v>La Liga</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Camp Nou</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Barcelona</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Spain</v>
+      </c>
+      <c r="F3">
+        <v>1957</v>
+      </c>
+      <c r="G3">
+        <v>99354</v>
+      </c>
+      <c r="H3">
+        <v>41.3815</v>
+      </c>
+      <c r="I3">
+        <v>2.1212</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Josep Soteras</v>
+      </c>
+      <c r="K3" t="str">
         <v>Grass</v>
       </c>
-      <c r="M2" t="str">
-        <v>#DA291C</v>
-      </c>
-      <c r="N2" t="str">
-        <v>#000000</v>
-      </c>
-      <c r="O2" t="str">
-        <v>#FDB913</v>
-      </c>
-      <c r="P2" t="str">
-        <v>Theatre of Dreams,Rich history,Manchester United</v>
-      </c>
-      <c r="Q2" t="str">
-        <v>First FA Cup win 1909|European dominance</v>
-      </c>
-      <c r="R2">
-        <v>34</v>
-      </c>
-      <c r="S2" t="str">
-        <v>Theatre of Dreams</v>
-      </c>
-      <c r="T2" t="str">
-        <v>Premier League|FA Cup|Champions League</v>
-      </c>
-      <c r="U2" t="str">
-        <v>Manchester United 20 titles</v>
-      </c>
-      <c r="V2">
-        <v>2</v>
+      <c r="L3" t="str">
+        <v>Camp of Wonders</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Barcelona FC,Capacity,Architecture</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Messi era|Champions League wins</v>
+      </c>
+      <c r="O3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Football</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Serie A</v>
+      </c>
+      <c r="C4" t="str">
+        <v>San Siro</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Milan</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Italy</v>
+      </c>
+      <c r="F4">
+        <v>1926</v>
+      </c>
+      <c r="G4">
+        <v>80018</v>
+      </c>
+      <c r="H4">
+        <v>45.4771</v>
+      </c>
+      <c r="I4">
+        <v>9.1289</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Armando Dazzi</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Grass</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Stadio Giuseppe Meazza</v>
+      </c>
+      <c r="M4" t="str">
+        <v>AC Milan,Inter Milan,Derby</v>
+      </c>
+      <c r="N4" t="str">
+        <v>European Cups|Derby matches</v>
+      </c>
+      <c r="O4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Football</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Premier League</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Wembley Stadium</v>
+      </c>
+      <c r="D5" t="str">
+        <v>London</v>
+      </c>
+      <c r="E5" t="str">
+        <v>England</v>
+      </c>
+      <c r="F5">
+        <v>2019</v>
+      </c>
+      <c r="G5">
+        <v>90000</v>
+      </c>
+      <c r="H5">
+        <v>51.5559</v>
+      </c>
+      <c r="I5">
+        <v>-0.2795</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Norman Foster</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Grass</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Home of Football</v>
+      </c>
+      <c r="M5" t="str">
+        <v>England home,1966 victory,Modern</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Euro 2020 final|England victories</v>
+      </c>
+      <c r="O5">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:O3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>sport</v>
+      </c>
+      <c r="B1" t="str">
+        <v>competition</v>
+      </c>
+      <c r="C1" t="str">
+        <v>venueName</v>
+      </c>
+      <c r="D1" t="str">
+        <v>city</v>
+      </c>
+      <c r="E1" t="str">
+        <v>country</v>
+      </c>
+      <c r="F1" t="str">
+        <v>opened</v>
+      </c>
+      <c r="G1" t="str">
+        <v>capacity</v>
+      </c>
+      <c r="H1" t="str">
+        <v>lat</v>
+      </c>
+      <c r="I1" t="str">
+        <v>lng</v>
+      </c>
+      <c r="J1" t="str">
+        <v>architect</v>
+      </c>
+      <c r="K1" t="str">
+        <v>surface</v>
+      </c>
+      <c r="L1" t="str">
+        <v>nickname</v>
+      </c>
+      <c r="M1" t="str">
+        <v>famousFor</v>
+      </c>
+      <c r="N1" t="str">
+        <v>iconicMoments</v>
+      </c>
+      <c r="O1" t="str">
+        <v>collectorNumber</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Cricket</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Test Cricket</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Lords Cricket Ground</v>
+      </c>
+      <c r="D2" t="str">
+        <v>London</v>
+      </c>
+      <c r="E2" t="str">
+        <v>England</v>
+      </c>
+      <c r="F2">
+        <v>1814</v>
+      </c>
+      <c r="G2">
+        <v>30000</v>
+      </c>
+      <c r="H2">
+        <v>51.5156</v>
+      </c>
+      <c r="I2">
+        <v>-0.1244</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Thomas Lord</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Grass</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Home of Cricket</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Historic,Tradition,MCC</v>
+      </c>
+      <c r="N2" t="str">
+        <v>First match 1877|Test cricket hub</v>
+      </c>
+      <c r="O2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Cricket</v>
+      </c>
+      <c r="B3" t="str">
+        <v>IPL</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Eden Gardens</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Kolkata</v>
+      </c>
+      <c r="E3" t="str">
+        <v>India</v>
+      </c>
+      <c r="F3">
+        <v>1934</v>
+      </c>
+      <c r="G3">
+        <v>68000</v>
+      </c>
+      <c r="H3">
+        <v>22.5651</v>
+      </c>
+      <c r="I3">
+        <v>88.3828</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Historic Design</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Grass</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Castle of Cricket</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Passionate crowds,Historic,India</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Test victories|IPL finals</v>
+      </c>
+      <c r="O3">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:O3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:O3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>sport</v>
+      </c>
+      <c r="B1" t="str">
+        <v>competition</v>
+      </c>
+      <c r="C1" t="str">
+        <v>venueName</v>
+      </c>
+      <c r="D1" t="str">
+        <v>city</v>
+      </c>
+      <c r="E1" t="str">
+        <v>country</v>
+      </c>
+      <c r="F1" t="str">
+        <v>opened</v>
+      </c>
+      <c r="G1" t="str">
+        <v>capacity</v>
+      </c>
+      <c r="H1" t="str">
+        <v>lat</v>
+      </c>
+      <c r="I1" t="str">
+        <v>lng</v>
+      </c>
+      <c r="J1" t="str">
+        <v>architect</v>
+      </c>
+      <c r="K1" t="str">
+        <v>surface</v>
+      </c>
+      <c r="L1" t="str">
+        <v>nickname</v>
+      </c>
+      <c r="M1" t="str">
+        <v>famousFor</v>
+      </c>
+      <c r="N1" t="str">
+        <v>iconicMoments</v>
+      </c>
+      <c r="O1" t="str">
+        <v>collectorNumber</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Tennis</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Wimbledon</v>
+      </c>
+      <c r="C2" t="str">
+        <v>All England Lawn Tennis Club</v>
+      </c>
+      <c r="D2" t="str">
+        <v>London</v>
+      </c>
+      <c r="E2" t="str">
+        <v>England</v>
+      </c>
+      <c r="F2">
+        <v>1877</v>
+      </c>
+      <c r="G2">
+        <v>15000</v>
+      </c>
+      <c r="H2">
+        <v>51.4347</v>
+      </c>
+      <c r="I2">
+        <v>-0.2157</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Historic Design</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Grass</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Mecca of Tennis</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Grand Slam,Grass courts,Tradition</v>
+      </c>
+      <c r="N2" t="str">
+        <v>First Grand Slam 1877|Murray 2013</v>
+      </c>
+      <c r="O2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Tennis</v>
+      </c>
+      <c r="B3" t="str">
+        <v>US Open</v>
+      </c>
+      <c r="C3" t="str">
+        <v>USTA National Tennis Center</v>
+      </c>
+      <c r="D3" t="str">
+        <v>New York</v>
+      </c>
+      <c r="E3" t="str">
+        <v>USA</v>
+      </c>
+      <c r="F3">
+        <v>1978</v>
+      </c>
+      <c r="G3">
+        <v>24000</v>
+      </c>
+      <c r="H3">
+        <v>40.7589</v>
+      </c>
+      <c r="I3">
+        <v>-73.8204</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Modern Design</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Hard court</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Arthur Ashe Stadium</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Grand Slam,Hard court,American</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Serena dominance|Nadal records</v>
+      </c>
+      <c r="O3">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:O3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:O3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>sport</v>
+      </c>
+      <c r="B1" t="str">
+        <v>competition</v>
+      </c>
+      <c r="C1" t="str">
+        <v>venueName</v>
+      </c>
+      <c r="D1" t="str">
+        <v>city</v>
+      </c>
+      <c r="E1" t="str">
+        <v>country</v>
+      </c>
+      <c r="F1" t="str">
+        <v>opened</v>
+      </c>
+      <c r="G1" t="str">
+        <v>capacity</v>
+      </c>
+      <c r="H1" t="str">
+        <v>lat</v>
+      </c>
+      <c r="I1" t="str">
+        <v>lng</v>
+      </c>
+      <c r="J1" t="str">
+        <v>architect</v>
+      </c>
+      <c r="K1" t="str">
+        <v>surface</v>
+      </c>
+      <c r="L1" t="str">
+        <v>nickname</v>
+      </c>
+      <c r="M1" t="str">
+        <v>famousFor</v>
+      </c>
+      <c r="N1" t="str">
+        <v>iconicMoments</v>
+      </c>
+      <c r="O1" t="str">
+        <v>collectorNumber</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Golf</v>
+      </c>
+      <c r="B2" t="str">
+        <v>The Open Championship</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Old Course at St Andrews</v>
+      </c>
+      <c r="D2" t="str">
+        <v>St Andrews</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Scotland</v>
+      </c>
+      <c r="F2">
+        <v>1552</v>
+      </c>
+      <c r="G2">
+        <v>40000</v>
+      </c>
+      <c r="H2">
+        <v>56.3903</v>
+      </c>
+      <c r="I2">
+        <v>-2.7933</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Natural course</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Links grass</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Home of Golf</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Oldest course,Historic,Links</v>
+      </c>
+      <c r="N2" t="str">
+        <v>First tournament 1873|Tiger wins</v>
+      </c>
+      <c r="O2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Golf</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Masters Tournament</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Augusta National Golf Club</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Augusta</v>
+      </c>
+      <c r="E3" t="str">
+        <v>USA</v>
+      </c>
+      <c r="F3">
+        <v>1933</v>
+      </c>
+      <c r="G3">
+        <v>30000</v>
+      </c>
+      <c r="H3">
+        <v>33.5028</v>
+      </c>
+      <c r="I3">
+        <v>-82.0138</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Bobby Jones</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Championship grass</v>
+      </c>
+      <c r="L3" t="str">
+        <v>The Masters</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Green jacket,Prestige,Tradition</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Tiger comeback 2019|Nicklaus era</v>
+      </c>
+      <c r="O3">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:O3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:O2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>sport</v>
+      </c>
+      <c r="B1" t="str">
+        <v>competition</v>
+      </c>
+      <c r="C1" t="str">
+        <v>venueName</v>
+      </c>
+      <c r="D1" t="str">
+        <v>city</v>
+      </c>
+      <c r="E1" t="str">
+        <v>country</v>
+      </c>
+      <c r="F1" t="str">
+        <v>opened</v>
+      </c>
+      <c r="G1" t="str">
+        <v>capacity</v>
+      </c>
+      <c r="H1" t="str">
+        <v>lat</v>
+      </c>
+      <c r="I1" t="str">
+        <v>lng</v>
+      </c>
+      <c r="J1" t="str">
+        <v>architect</v>
+      </c>
+      <c r="K1" t="str">
+        <v>surface</v>
+      </c>
+      <c r="L1" t="str">
+        <v>nickname</v>
+      </c>
+      <c r="M1" t="str">
+        <v>famousFor</v>
+      </c>
+      <c r="N1" t="str">
+        <v>iconicMoments</v>
+      </c>
+      <c r="O1" t="str">
+        <v>collectorNumber</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Rugby</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Six Nations</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Twickenham Stadium</v>
+      </c>
+      <c r="D2" t="str">
+        <v>London</v>
+      </c>
+      <c r="E2" t="str">
+        <v>England</v>
+      </c>
+      <c r="F2">
+        <v>1907</v>
+      </c>
+      <c r="G2">
+        <v>82000</v>
+      </c>
+      <c r="H2">
+        <v>51.4545</v>
+      </c>
+      <c r="I2">
+        <v>-0.3394</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Archibald Leitch</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Grass</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Fortress England</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Rugby HQ,Historic,England home</v>
+      </c>
+      <c r="N2" t="str">
+        <v>1999 World Cup|England Grand Slams</v>
+      </c>
+      <c r="O2">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:O2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>sport</v>
+      </c>
+      <c r="B1" t="str">
+        <v>competition</v>
+      </c>
+      <c r="C1" t="str">
+        <v>venueName</v>
+      </c>
+      <c r="D1" t="str">
+        <v>city</v>
+      </c>
+      <c r="E1" t="str">
+        <v>country</v>
+      </c>
+      <c r="F1" t="str">
+        <v>opened</v>
+      </c>
+      <c r="G1" t="str">
+        <v>capacity</v>
+      </c>
+      <c r="H1" t="str">
+        <v>lat</v>
+      </c>
+      <c r="I1" t="str">
+        <v>lng</v>
+      </c>
+      <c r="J1" t="str">
+        <v>architect</v>
+      </c>
+      <c r="K1" t="str">
+        <v>surface</v>
+      </c>
+      <c r="L1" t="str">
+        <v>nickname</v>
+      </c>
+      <c r="M1" t="str">
+        <v>famousFor</v>
+      </c>
+      <c r="N1" t="str">
+        <v>iconicMoments</v>
+      </c>
+      <c r="O1" t="str">
+        <v>collectorNumber</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Olympic Venues</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Summer Olympics</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Estadio Nacional de Beijing</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Beijing</v>
+      </c>
+      <c r="E2" t="str">
+        <v>China</v>
+      </c>
+      <c r="F2">
+        <v>2008</v>
+      </c>
+      <c r="G2">
+        <v>91000</v>
+      </c>
+      <c r="H2">
+        <v>39.9942</v>
+      </c>
+      <c r="I2">
+        <v>116.4074</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Herzog and de Meuron</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Track and field</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Bird's Nest</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Architecture,Beijing 2008,Modern</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Bolt records|Phelps 8 golds</v>
+      </c>
+      <c r="O2">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:O2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>sport</v>
+      </c>
+      <c r="B1" t="str">
+        <v>competition</v>
+      </c>
+      <c r="C1" t="str">
+        <v>venueName</v>
+      </c>
+      <c r="D1" t="str">
+        <v>city</v>
+      </c>
+      <c r="E1" t="str">
+        <v>country</v>
+      </c>
+      <c r="F1" t="str">
+        <v>opened</v>
+      </c>
+      <c r="G1" t="str">
+        <v>capacity</v>
+      </c>
+      <c r="H1" t="str">
+        <v>lat</v>
+      </c>
+      <c r="I1" t="str">
+        <v>lng</v>
+      </c>
+      <c r="J1" t="str">
+        <v>architect</v>
+      </c>
+      <c r="K1" t="str">
+        <v>surface</v>
+      </c>
+      <c r="L1" t="str">
+        <v>nickname</v>
+      </c>
+      <c r="M1" t="str">
+        <v>famousFor</v>
+      </c>
+      <c r="N1" t="str">
+        <v>iconicMoments</v>
+      </c>
+      <c r="O1" t="str">
+        <v>collectorNumber</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Boxing</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Title Fights</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Madison Square Garden</v>
+      </c>
+      <c r="D2" t="str">
+        <v>New York</v>
+      </c>
+      <c r="E2" t="str">
+        <v>USA</v>
+      </c>
+      <c r="F2">
+        <v>1968</v>
+      </c>
+      <c r="G2">
+        <v>20000</v>
+      </c>
+      <c r="H2">
+        <v>40.7505</v>
+      </c>
+      <c r="I2">
+        <v>-73.9934</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Modern Design</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Indoor arena</v>
+      </c>
+      <c r="L2" t="str">
+        <v>The Garden</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Boxing history,Title fights,Iconic</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Ali vs Frazier 1971|Tyson fights</v>
+      </c>
+      <c r="O2">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>